<commit_message>
Add image transformation and about window
</commit_message>
<xml_diff>
--- a/app/database/MSI_database_V1.0_small.xlsx
+++ b/app/database/MSI_database_V1.0_small.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0065634/Documents/Software_projects/msi-quant/app/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2132B4-FF88-624C-B273-C981715E1CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{721A74C0-AF42-3A4C-9A0C-791A1B4B2268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3000" yWindow="500" windowWidth="31520" windowHeight="19080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="150">
   <si>
     <t>ID</t>
   </si>
@@ -89,9 +89,6 @@
     <t>Na+ Isotope</t>
   </si>
   <si>
-    <t>[M+H]+,[M+Na]+,[M+K]+</t>
-  </si>
-  <si>
     <t>Adducts</t>
   </si>
   <si>
@@ -485,121 +482,7 @@
     <t>C52H80NPO8</t>
   </si>
   <si>
-    <t>LPC 14:0</t>
-  </si>
-  <si>
-    <t>LPC 16:0</t>
-  </si>
-  <si>
-    <t>LPC 18:0</t>
-  </si>
-  <si>
-    <t>LPC 20:0</t>
-  </si>
-  <si>
-    <t>LPC 14:1</t>
-  </si>
-  <si>
-    <t>LPC 16:1</t>
-  </si>
-  <si>
-    <t>LPC 18:1</t>
-  </si>
-  <si>
-    <t>LPC 20:1</t>
-  </si>
-  <si>
-    <t>LPC 22:1</t>
-  </si>
-  <si>
-    <t>LPC 18:2</t>
-  </si>
-  <si>
-    <t>LPC 20:2</t>
-  </si>
-  <si>
-    <t>LPC 18:3</t>
-  </si>
-  <si>
-    <t>LPC 20:3</t>
-  </si>
-  <si>
-    <t>LPC 18:4</t>
-  </si>
-  <si>
-    <t>LPC 20:4</t>
-  </si>
-  <si>
-    <t>LPC 22:4</t>
-  </si>
-  <si>
-    <t>LPC 20:5</t>
-  </si>
-  <si>
-    <t>LPC 22:5</t>
-  </si>
-  <si>
-    <t>LPC 22:6</t>
-  </si>
-  <si>
-    <t>LPC</t>
-  </si>
-  <si>
-    <t>C22H46NPO7</t>
-  </si>
-  <si>
-    <t>C24H50NPO7</t>
-  </si>
-  <si>
-    <t>C26H54NPO7</t>
-  </si>
-  <si>
-    <t>C28H58NPO7</t>
-  </si>
-  <si>
-    <t>C22H44NPO7</t>
-  </si>
-  <si>
-    <t>C24H48NPO7</t>
-  </si>
-  <si>
-    <t>C26H52NPO7</t>
-  </si>
-  <si>
-    <t>C28H56NPO7</t>
-  </si>
-  <si>
-    <t>C30H60NPO7</t>
-  </si>
-  <si>
-    <t>C26H50NPO7</t>
-  </si>
-  <si>
-    <t>C28H54NPO7</t>
-  </si>
-  <si>
-    <t>C26H48NPO7</t>
-  </si>
-  <si>
-    <t>C28H52NPO7</t>
-  </si>
-  <si>
-    <t>C26H46NPO7</t>
-  </si>
-  <si>
-    <t>C28H50NPO7</t>
-  </si>
-  <si>
-    <t>C30H54NPO7</t>
-  </si>
-  <si>
-    <t>C28H48NPO7</t>
-  </si>
-  <si>
-    <t>C30H52NPO7</t>
-  </si>
-  <si>
-    <t>C30H50NPO7</t>
+    <t>[M+H]+,[M+K]+</t>
   </si>
 </sst>
 </file>
@@ -973,7 +856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.5" bestFit="1" customWidth="1"/>
@@ -995,10 +878,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>16</v>
@@ -1024,10 +907,10 @@
         <v>2</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -1041,19 +924,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" t="s">
@@ -1065,19 +948,19 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" t="s">
@@ -1089,16 +972,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F5" t="s">
         <v>3</v>
@@ -1113,16 +996,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F6" t="s">
         <v>4</v>
@@ -1137,16 +1020,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F7" t="s">
         <v>5</v>
@@ -1161,19 +1044,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
         <v>2</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E8" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" t="s">
@@ -1185,19 +1068,19 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
         <v>2</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" t="s">
@@ -1209,19 +1092,19 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
         <v>2</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E10" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" t="s">
@@ -1233,19 +1116,19 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
         <v>2</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E11" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" t="s">
@@ -1263,10 +1146,10 @@
         <v>2</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E12" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -1287,10 +1170,10 @@
         <v>2</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E13" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F13" t="s">
         <v>7</v>
@@ -1311,10 +1194,10 @@
         <v>2</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F14" t="s">
         <v>8</v>
@@ -1328,19 +1211,19 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
         <v>2</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E15" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I15" t="s">
         <v>9</v>
@@ -1351,19 +1234,19 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
         <v>2</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E16" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I16" t="s">
         <v>9</v>
@@ -1374,19 +1257,19 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
         <v>2</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E17" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I17" t="s">
         <v>9</v>
@@ -1397,16 +1280,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
         <v>2</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E18" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="I18" t="s">
         <v>9</v>
@@ -1417,16 +1300,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
         <v>2</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E19" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="I19" t="s">
         <v>9</v>
@@ -1443,13 +1326,13 @@
         <v>2</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I20" t="s">
         <v>9</v>
@@ -1466,13 +1349,13 @@
         <v>2</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E21" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I21" t="s">
         <v>9</v>
@@ -1489,13 +1372,13 @@
         <v>2</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E22" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I22" t="s">
         <v>9</v>
@@ -1506,19 +1389,19 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C23" t="s">
         <v>2</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E23" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F23" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I23" t="s">
         <v>9</v>
@@ -1529,19 +1412,19 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C24" t="s">
         <v>2</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E24" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I24" t="s">
         <v>9</v>
@@ -1552,19 +1435,19 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C25" t="s">
         <v>2</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E25" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I25" t="s">
         <v>9</v>
@@ -1575,16 +1458,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C26" t="s">
         <v>2</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E26" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="I26" t="s">
         <v>9</v>
@@ -1595,22 +1478,22 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C27" t="s">
         <v>2</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E27" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F27" t="s">
         <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I27" t="s">
         <v>9</v>
@@ -1621,22 +1504,22 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
         <v>2</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E28" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F28" t="s">
         <v>11</v>
       </c>
       <c r="G28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I28" t="s">
         <v>9</v>
@@ -1647,22 +1530,22 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C29" t="s">
         <v>2</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E29" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F29" t="s">
         <v>12</v>
       </c>
       <c r="G29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I29" t="s">
         <v>9</v>
@@ -1673,22 +1556,22 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C30" t="s">
         <v>2</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E30" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F30" t="s">
         <v>13</v>
       </c>
       <c r="G30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I30" t="s">
         <v>9</v>
@@ -1699,22 +1582,22 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C31" t="s">
         <v>2</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E31" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I31" t="s">
         <v>9</v>
@@ -1725,22 +1608,22 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C32" t="s">
         <v>2</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E32" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I32" t="s">
         <v>9</v>
@@ -1757,16 +1640,16 @@
         <v>2</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E33" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F33" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G33" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I33" t="s">
         <v>9</v>
@@ -1783,13 +1666,13 @@
         <v>2</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E34" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G34" t="s">
         <v>3</v>
@@ -1809,13 +1692,13 @@
         <v>2</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E35" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G35" t="s">
         <v>4</v>
@@ -1835,13 +1718,13 @@
         <v>2</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E36" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G36" t="s">
         <v>5</v>
@@ -1855,22 +1738,22 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C37" t="s">
         <v>2</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E37" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I37" t="s">
         <v>9</v>
@@ -1881,22 +1764,22 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C38" t="s">
         <v>2</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E38" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I38" t="s">
         <v>9</v>
@@ -1907,19 +1790,19 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C39" t="s">
         <v>2</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E39" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="G39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I39" t="s">
         <v>9</v>
@@ -1930,19 +1813,19 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C40" t="s">
         <v>2</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E40" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G40" t="s">
         <v>6</v>
@@ -1956,19 +1839,19 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C41" t="s">
         <v>2</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E41" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G41" t="s">
         <v>7</v>
@@ -1982,19 +1865,19 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C42" t="s">
         <v>2</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E42" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F42" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G42" t="s">
         <v>8</v>
@@ -2008,22 +1891,22 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C43" t="s">
         <v>2</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E43" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I43" t="s">
         <v>9</v>
@@ -2034,22 +1917,22 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C44" t="s">
         <v>2</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E44" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F44" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I44" t="s">
         <v>9</v>
@@ -2060,22 +1943,22 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C45" t="s">
         <v>2</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E45" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I45" t="s">
         <v>9</v>
@@ -2086,19 +1969,19 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C46" t="s">
         <v>2</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E46" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="G46" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I46" t="s">
         <v>9</v>
@@ -2109,22 +1992,22 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C47" t="s">
         <v>2</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E47" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I47" t="s">
         <v>9</v>
@@ -2135,22 +2018,22 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C48" t="s">
         <v>2</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E48" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F48" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I48" t="s">
         <v>9</v>
@@ -2161,22 +2044,22 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C49" t="s">
         <v>2</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E49" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F49" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I49" t="s">
         <v>9</v>
@@ -2187,22 +2070,22 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C50" t="s">
         <v>2</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E50" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F50" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G50" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I50" t="s">
         <v>9</v>
@@ -2213,22 +2096,22 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C51" t="s">
         <v>2</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E51" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F51" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G51" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I51" t="s">
         <v>9</v>
@@ -2239,19 +2122,19 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C52" t="s">
         <v>2</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E52" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G52" t="s">
         <v>11</v>
@@ -2265,19 +2148,19 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C53" t="s">
         <v>2</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E53" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F53" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G53" t="s">
         <v>12</v>
@@ -2291,19 +2174,19 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C54" t="s">
         <v>2</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E54" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F54" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G54" t="s">
         <v>13</v>
@@ -2317,22 +2200,22 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C55" t="s">
         <v>2</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E55" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F55" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G55" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I55" t="s">
         <v>9</v>
@@ -2343,22 +2226,22 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C56" t="s">
         <v>2</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E56" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G56" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I56" t="s">
         <v>9</v>
@@ -2369,19 +2252,19 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C57" t="s">
         <v>2</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E57" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="G57" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I57" t="s">
         <v>9</v>
@@ -2392,22 +2275,22 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C58" t="s">
         <v>2</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E58" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G58" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I58" t="s">
         <v>9</v>
@@ -2418,22 +2301,22 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C59" t="s">
         <v>2</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E59" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F59" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G59" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I59" t="s">
         <v>9</v>
@@ -2444,22 +2327,22 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C60" t="s">
         <v>2</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E60" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F60" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I60" t="s">
         <v>9</v>
@@ -2470,22 +2353,22 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C61" t="s">
         <v>2</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E61" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F61" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G61" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I61" t="s">
         <v>9</v>
@@ -2496,19 +2379,19 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C62" t="s">
         <v>2</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E62" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="G62" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I62" t="s">
         <v>9</v>
@@ -2519,22 +2402,22 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C63" t="s">
         <v>2</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E63" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F63" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G63" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I63" t="s">
         <v>9</v>
@@ -2545,22 +2428,22 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C64" t="s">
         <v>2</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E64" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F64" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G64" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I64" t="s">
         <v>9</v>
@@ -2571,22 +2454,22 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C65" t="s">
         <v>2</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E65" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F65" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G65" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I65" t="s">
         <v>9</v>
@@ -2597,19 +2480,19 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C66" t="s">
         <v>2</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E66" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="G66" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I66" t="s">
         <v>9</v>
@@ -2620,22 +2503,22 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C67" t="s">
         <v>2</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E67" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F67" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G67" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I67" t="s">
         <v>9</v>
@@ -2646,22 +2529,22 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C68" t="s">
         <v>2</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E68" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="F68" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I68" t="s">
         <v>9</v>
@@ -2672,19 +2555,19 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C69" t="s">
         <v>2</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E69" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="G69" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I69" t="s">
         <v>9</v>
@@ -2695,22 +2578,22 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
+        <v>88</v>
+      </c>
+      <c r="C70" t="s">
+        <v>2</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="E70" t="s">
+        <v>149</v>
+      </c>
+      <c r="F70" t="s">
         <v>89</v>
       </c>
-      <c r="C70" t="s">
-        <v>2</v>
-      </c>
-      <c r="D70" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="E70" t="s">
-        <v>18</v>
-      </c>
-      <c r="F70" t="s">
-        <v>90</v>
-      </c>
       <c r="G70" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I70" t="s">
         <v>9</v>
@@ -2721,408 +2604,22 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C71" t="s">
         <v>2</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E71" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="G71" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I71" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A72" s="3">
-        <v>70</v>
-      </c>
-      <c r="B72" t="s">
-        <v>150</v>
-      </c>
-      <c r="C72" t="s">
-        <v>169</v>
-      </c>
-      <c r="D72" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="E72" t="s">
-        <v>18</v>
-      </c>
-      <c r="F72" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A73" s="1">
-        <v>71</v>
-      </c>
-      <c r="B73" t="s">
-        <v>151</v>
-      </c>
-      <c r="C73" t="s">
-        <v>169</v>
-      </c>
-      <c r="D73" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="E73" t="s">
-        <v>18</v>
-      </c>
-      <c r="F73" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A74" s="3">
-        <v>72</v>
-      </c>
-      <c r="B74" t="s">
-        <v>152</v>
-      </c>
-      <c r="C74" t="s">
-        <v>169</v>
-      </c>
-      <c r="D74" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="E74" t="s">
-        <v>18</v>
-      </c>
-      <c r="F74" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A75" s="1">
-        <v>73</v>
-      </c>
-      <c r="B75" t="s">
-        <v>153</v>
-      </c>
-      <c r="C75" t="s">
-        <v>169</v>
-      </c>
-      <c r="D75" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="E75" t="s">
-        <v>18</v>
-      </c>
-      <c r="F75" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A76" s="3">
-        <v>74</v>
-      </c>
-      <c r="B76" t="s">
-        <v>154</v>
-      </c>
-      <c r="C76" t="s">
-        <v>169</v>
-      </c>
-      <c r="D76" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="E76" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A77" s="1">
-        <v>75</v>
-      </c>
-      <c r="B77" t="s">
-        <v>155</v>
-      </c>
-      <c r="C77" t="s">
-        <v>169</v>
-      </c>
-      <c r="D77" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="E77" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A78" s="3">
-        <v>76</v>
-      </c>
-      <c r="B78" t="s">
-        <v>156</v>
-      </c>
-      <c r="C78" t="s">
-        <v>169</v>
-      </c>
-      <c r="D78" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="E78" t="s">
-        <v>18</v>
-      </c>
-      <c r="F78" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A79" s="1">
-        <v>77</v>
-      </c>
-      <c r="B79" t="s">
-        <v>157</v>
-      </c>
-      <c r="C79" t="s">
-        <v>169</v>
-      </c>
-      <c r="D79" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="E79" t="s">
-        <v>18</v>
-      </c>
-      <c r="F79" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A80" s="3">
-        <v>78</v>
-      </c>
-      <c r="B80" t="s">
-        <v>158</v>
-      </c>
-      <c r="C80" t="s">
-        <v>169</v>
-      </c>
-      <c r="D80" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="E80" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A81" s="1">
-        <v>79</v>
-      </c>
-      <c r="B81" t="s">
-        <v>159</v>
-      </c>
-      <c r="C81" t="s">
-        <v>169</v>
-      </c>
-      <c r="D81" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="E81" t="s">
-        <v>18</v>
-      </c>
-      <c r="F81" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A82" s="3">
-        <v>80</v>
-      </c>
-      <c r="B82" t="s">
-        <v>160</v>
-      </c>
-      <c r="C82" t="s">
-        <v>169</v>
-      </c>
-      <c r="D82" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="E82" t="s">
-        <v>18</v>
-      </c>
-      <c r="F82" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A83" s="1">
-        <v>81</v>
-      </c>
-      <c r="B83" t="s">
-        <v>161</v>
-      </c>
-      <c r="C83" t="s">
-        <v>169</v>
-      </c>
-      <c r="D83" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="E83" t="s">
-        <v>18</v>
-      </c>
-      <c r="F83" t="s">
-        <v>163</v>
-      </c>
-      <c r="G83" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A84" s="3">
-        <v>82</v>
-      </c>
-      <c r="B84" t="s">
-        <v>162</v>
-      </c>
-      <c r="C84" t="s">
-        <v>169</v>
-      </c>
-      <c r="D84" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="E84" t="s">
-        <v>18</v>
-      </c>
-      <c r="F84" t="s">
-        <v>164</v>
-      </c>
-      <c r="G84" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A85" s="1">
-        <v>83</v>
-      </c>
-      <c r="B85" t="s">
-        <v>163</v>
-      </c>
-      <c r="C85" t="s">
-        <v>169</v>
-      </c>
-      <c r="D85" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="E85" t="s">
-        <v>18</v>
-      </c>
-      <c r="G85" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A86" s="3">
-        <v>84</v>
-      </c>
-      <c r="B86" t="s">
-        <v>164</v>
-      </c>
-      <c r="C86" t="s">
-        <v>169</v>
-      </c>
-      <c r="D86" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="E86" t="s">
-        <v>18</v>
-      </c>
-      <c r="F86" t="s">
-        <v>166</v>
-      </c>
-      <c r="G86" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A87" s="1">
-        <v>85</v>
-      </c>
-      <c r="B87" t="s">
-        <v>165</v>
-      </c>
-      <c r="C87" t="s">
-        <v>169</v>
-      </c>
-      <c r="D87" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="E87" t="s">
-        <v>18</v>
-      </c>
-      <c r="F87" t="s">
-        <v>167</v>
-      </c>
-      <c r="G87" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A88" s="3">
-        <v>86</v>
-      </c>
-      <c r="B88" t="s">
-        <v>166</v>
-      </c>
-      <c r="C88" t="s">
-        <v>169</v>
-      </c>
-      <c r="D88" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="E88" t="s">
-        <v>18</v>
-      </c>
-      <c r="G88" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A89" s="1">
-        <v>87</v>
-      </c>
-      <c r="B89" t="s">
-        <v>167</v>
-      </c>
-      <c r="C89" t="s">
-        <v>169</v>
-      </c>
-      <c r="D89" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="E89" t="s">
-        <v>18</v>
-      </c>
-      <c r="F89" t="s">
-        <v>168</v>
-      </c>
-      <c r="G89" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A90" s="3">
-        <v>88</v>
-      </c>
-      <c r="B90" t="s">
-        <v>168</v>
-      </c>
-      <c r="C90" t="s">
-        <v>169</v>
-      </c>
-      <c r="D90" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="E90" t="s">
-        <v>18</v>
-      </c>
-      <c r="G90" t="s">
-        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move user editable files outside app
</commit_message>
<xml_diff>
--- a/app/database/MSI_database_V1.0_small.xlsx
+++ b/app/database/MSI_database_V1.0_small.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0065634/Documents/Software_projects/LipidQMap/app/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07EAC78D-6D82-134C-B0BF-00E734DD1879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14DB6DA7-3C17-4A49-B5F9-4DF83DBC5185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="152">
   <si>
     <t>ID</t>
   </si>
@@ -473,6 +473,9 @@
   </si>
   <si>
     <t>M-4 Isotope</t>
+  </si>
+  <si>
+    <t>IS standard</t>
   </si>
 </sst>
 </file>
@@ -836,10 +839,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -862,13 +865,16 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -881,11 +887,14 @@
       <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2">
         <v>1.5</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -901,11 +910,14 @@
       <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="I3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -921,11 +933,14 @@
       <c r="E4" t="s">
         <v>17</v>
       </c>
-      <c r="I4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -941,11 +956,14 @@
       <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="I5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -961,11 +979,14 @@
       <c r="E6" t="s">
         <v>23</v>
       </c>
-      <c r="I6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -981,11 +1002,14 @@
       <c r="E7" t="s">
         <v>26</v>
       </c>
-      <c r="I7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1001,11 +1025,14 @@
       <c r="E8" t="s">
         <v>29</v>
       </c>
-      <c r="I8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1021,11 +1048,14 @@
       <c r="E9" t="s">
         <v>32</v>
       </c>
-      <c r="I9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1041,11 +1071,14 @@
       <c r="E10" t="s">
         <v>34</v>
       </c>
-      <c r="I10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1061,11 +1094,14 @@
       <c r="E11" t="s">
         <v>36</v>
       </c>
-      <c r="I11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1081,11 +1117,14 @@
       <c r="E12" t="s">
         <v>38</v>
       </c>
-      <c r="I12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -1101,11 +1140,14 @@
       <c r="E13" t="s">
         <v>40</v>
       </c>
-      <c r="I13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1121,11 +1163,14 @@
       <c r="E14" t="s">
         <v>42</v>
       </c>
-      <c r="I14" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1141,11 +1186,14 @@
       <c r="E15" t="s">
         <v>44</v>
       </c>
-      <c r="I15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1161,11 +1209,14 @@
       <c r="E16" t="s">
         <v>46</v>
       </c>
-      <c r="I16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H16" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>47</v>
       </c>
@@ -1181,11 +1232,14 @@
       <c r="E17" t="s">
         <v>49</v>
       </c>
-      <c r="I17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1198,11 +1252,14 @@
       <c r="D18" t="s">
         <v>11</v>
       </c>
-      <c r="I18" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H18" t="b">
+        <v>1</v>
+      </c>
+      <c r="J18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -1215,11 +1272,14 @@
       <c r="D19" t="s">
         <v>11</v>
       </c>
-      <c r="I19" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -1235,11 +1295,14 @@
       <c r="E20" t="s">
         <v>53</v>
       </c>
-      <c r="I20" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="J20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -1255,11 +1318,14 @@
       <c r="E21" t="s">
         <v>55</v>
       </c>
-      <c r="I21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="J21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -1275,11 +1341,14 @@
       <c r="E22" t="s">
         <v>57</v>
       </c>
-      <c r="I22" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H22" t="b">
+        <v>1</v>
+      </c>
+      <c r="J22" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -1295,11 +1364,14 @@
       <c r="E23" t="s">
         <v>59</v>
       </c>
-      <c r="I23" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="J23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -1315,11 +1387,14 @@
       <c r="E24" t="s">
         <v>61</v>
       </c>
-      <c r="I24" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H24" t="b">
+        <v>1</v>
+      </c>
+      <c r="J24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -1335,11 +1410,14 @@
       <c r="E25" t="s">
         <v>63</v>
       </c>
-      <c r="I25" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H25" t="b">
+        <v>1</v>
+      </c>
+      <c r="J25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -1352,11 +1430,14 @@
       <c r="D26" t="s">
         <v>11</v>
       </c>
-      <c r="I26" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H26" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -1375,11 +1456,14 @@
       <c r="G27" t="s">
         <v>15</v>
       </c>
-      <c r="I27" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H27" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>55</v>
       </c>
@@ -1398,11 +1482,14 @@
       <c r="G28" t="s">
         <v>18</v>
       </c>
-      <c r="I28" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H28" t="b">
+        <v>1</v>
+      </c>
+      <c r="J28" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>57</v>
       </c>
@@ -1421,11 +1508,14 @@
       <c r="G29" t="s">
         <v>21</v>
       </c>
-      <c r="I29" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
+      <c r="J29" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>59</v>
       </c>
@@ -1444,11 +1534,14 @@
       <c r="G30" t="s">
         <v>24</v>
       </c>
-      <c r="I30" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H30" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -1467,11 +1560,14 @@
       <c r="G31" t="s">
         <v>27</v>
       </c>
-      <c r="I31" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H31" t="b">
+        <v>1</v>
+      </c>
+      <c r="J31" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -1490,11 +1586,14 @@
       <c r="G32" t="s">
         <v>30</v>
       </c>
-      <c r="I32" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H32" t="b">
+        <v>1</v>
+      </c>
+      <c r="J32" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>67</v>
       </c>
@@ -1513,11 +1612,14 @@
       <c r="G33" t="s">
         <v>17</v>
       </c>
-      <c r="I33" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H33" t="b">
+        <v>1</v>
+      </c>
+      <c r="J33" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -1536,11 +1638,14 @@
       <c r="G34" t="s">
         <v>20</v>
       </c>
-      <c r="I34" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H34" t="b">
+        <v>1</v>
+      </c>
+      <c r="J34" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>71</v>
       </c>
@@ -1559,11 +1664,14 @@
       <c r="G35" t="s">
         <v>23</v>
       </c>
-      <c r="I35" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J35" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -1582,11 +1690,14 @@
       <c r="G36" t="s">
         <v>26</v>
       </c>
-      <c r="I36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H36" t="b">
+        <v>1</v>
+      </c>
+      <c r="J36" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -1605,11 +1716,14 @@
       <c r="G37" t="s">
         <v>29</v>
       </c>
-      <c r="I37" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H37" t="b">
+        <v>1</v>
+      </c>
+      <c r="J37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>77</v>
       </c>
@@ -1628,11 +1742,14 @@
       <c r="G38" t="s">
         <v>32</v>
       </c>
-      <c r="I38" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H38" t="b">
+        <v>1</v>
+      </c>
+      <c r="J38" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>79</v>
       </c>
@@ -1648,11 +1765,14 @@
       <c r="G39" t="s">
         <v>36</v>
       </c>
-      <c r="I39" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H39" t="b">
+        <v>1</v>
+      </c>
+      <c r="J39" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>81</v>
       </c>
@@ -1671,11 +1791,14 @@
       <c r="G40" t="s">
         <v>38</v>
       </c>
-      <c r="I40" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H40" t="b">
+        <v>1</v>
+      </c>
+      <c r="J40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>83</v>
       </c>
@@ -1694,11 +1817,14 @@
       <c r="G41" t="s">
         <v>40</v>
       </c>
-      <c r="I41" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H41" t="b">
+        <v>1</v>
+      </c>
+      <c r="J41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>85</v>
       </c>
@@ -1717,11 +1843,14 @@
       <c r="G42" t="s">
         <v>42</v>
       </c>
-      <c r="I42" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H42" t="b">
+        <v>1</v>
+      </c>
+      <c r="J42" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>87</v>
       </c>
@@ -1740,11 +1869,14 @@
       <c r="G43" t="s">
         <v>44</v>
       </c>
-      <c r="I43" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H43" t="b">
+        <v>1</v>
+      </c>
+      <c r="J43" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>89</v>
       </c>
@@ -1763,11 +1895,14 @@
       <c r="G44" t="s">
         <v>46</v>
       </c>
-      <c r="I44" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H44" t="b">
+        <v>1</v>
+      </c>
+      <c r="J44" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>101</v>
       </c>
@@ -1786,11 +1921,14 @@
       <c r="G45" t="s">
         <v>49</v>
       </c>
-      <c r="I45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H45" t="b">
+        <v>1</v>
+      </c>
+      <c r="J45" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>92</v>
       </c>
@@ -1806,11 +1944,14 @@
       <c r="G46" t="s">
         <v>53</v>
       </c>
-      <c r="I46" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H46" t="b">
+        <v>1</v>
+      </c>
+      <c r="J46" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>94</v>
       </c>
@@ -1829,11 +1970,14 @@
       <c r="G47" t="s">
         <v>55</v>
       </c>
-      <c r="I47" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H47" t="b">
+        <v>1</v>
+      </c>
+      <c r="J47" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>96</v>
       </c>
@@ -1852,11 +1996,14 @@
       <c r="G48" t="s">
         <v>57</v>
       </c>
-      <c r="I48" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H48" t="b">
+        <v>1</v>
+      </c>
+      <c r="J48" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>98</v>
       </c>
@@ -1875,11 +2022,14 @@
       <c r="G49" t="s">
         <v>59</v>
       </c>
-      <c r="I49" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H49" t="b">
+        <v>1</v>
+      </c>
+      <c r="J49" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>100</v>
       </c>
@@ -1898,11 +2048,14 @@
       <c r="G50" t="s">
         <v>61</v>
       </c>
-      <c r="I50" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H50" t="b">
+        <v>1</v>
+      </c>
+      <c r="J50" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>103</v>
       </c>
@@ -1921,11 +2074,14 @@
       <c r="G51" t="s">
         <v>63</v>
       </c>
-      <c r="I51" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H51" t="b">
+        <v>1</v>
+      </c>
+      <c r="J51" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>106</v>
       </c>
@@ -1944,11 +2100,14 @@
       <c r="G52" t="s">
         <v>69</v>
       </c>
-      <c r="I52" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H52" t="b">
+        <v>1</v>
+      </c>
+      <c r="J52" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>108</v>
       </c>
@@ -1967,11 +2126,14 @@
       <c r="G53" t="s">
         <v>71</v>
       </c>
-      <c r="I53" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H53" t="b">
+        <v>1</v>
+      </c>
+      <c r="J53" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>110</v>
       </c>
@@ -1990,11 +2152,14 @@
       <c r="G54" t="s">
         <v>73</v>
       </c>
-      <c r="I54" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H54" t="b">
+        <v>1</v>
+      </c>
+      <c r="J54" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>112</v>
       </c>
@@ -2013,11 +2178,14 @@
       <c r="G55" t="s">
         <v>75</v>
       </c>
-      <c r="I55" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H55" t="b">
+        <v>1</v>
+      </c>
+      <c r="J55" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>114</v>
       </c>
@@ -2036,11 +2204,14 @@
       <c r="G56" t="s">
         <v>77</v>
       </c>
-      <c r="I56" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H56" t="b">
+        <v>1</v>
+      </c>
+      <c r="J56" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>116</v>
       </c>
@@ -2056,11 +2227,14 @@
       <c r="G57" t="s">
         <v>81</v>
       </c>
-      <c r="I57" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H57" t="b">
+        <v>1</v>
+      </c>
+      <c r="J57" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>118</v>
       </c>
@@ -2079,11 +2253,14 @@
       <c r="G58" t="s">
         <v>83</v>
       </c>
-      <c r="I58" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H58" t="b">
+        <v>1</v>
+      </c>
+      <c r="J58" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>120</v>
       </c>
@@ -2102,11 +2279,14 @@
       <c r="G59" t="s">
         <v>85</v>
       </c>
-      <c r="I59" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H59" t="b">
+        <v>1</v>
+      </c>
+      <c r="J59" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>122</v>
       </c>
@@ -2125,11 +2305,14 @@
       <c r="G60" t="s">
         <v>87</v>
       </c>
-      <c r="I60" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H60" t="b">
+        <v>1</v>
+      </c>
+      <c r="J60" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>124</v>
       </c>
@@ -2148,11 +2331,14 @@
       <c r="G61" t="s">
         <v>89</v>
       </c>
-      <c r="I61" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H61" t="b">
+        <v>1</v>
+      </c>
+      <c r="J61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>127</v>
       </c>
@@ -2168,11 +2354,14 @@
       <c r="G62" t="s">
         <v>94</v>
       </c>
-      <c r="I62" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H62" t="b">
+        <v>1</v>
+      </c>
+      <c r="J62" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>129</v>
       </c>
@@ -2191,11 +2380,14 @@
       <c r="G63" t="s">
         <v>96</v>
       </c>
-      <c r="I63" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H63" t="b">
+        <v>1</v>
+      </c>
+      <c r="J63" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>131</v>
       </c>
@@ -2214,11 +2406,14 @@
       <c r="G64" t="s">
         <v>98</v>
       </c>
-      <c r="I64" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H64" t="b">
+        <v>1</v>
+      </c>
+      <c r="J64" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>133</v>
       </c>
@@ -2237,11 +2432,14 @@
       <c r="G65" t="s">
         <v>100</v>
       </c>
-      <c r="I65" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H65" t="b">
+        <v>1</v>
+      </c>
+      <c r="J65" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>136</v>
       </c>
@@ -2257,11 +2455,14 @@
       <c r="G66" t="s">
         <v>108</v>
       </c>
-      <c r="I66" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H66" t="b">
+        <v>1</v>
+      </c>
+      <c r="J66" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>138</v>
       </c>
@@ -2280,11 +2481,14 @@
       <c r="G67" t="s">
         <v>110</v>
       </c>
-      <c r="I67" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H67" t="b">
+        <v>1</v>
+      </c>
+      <c r="J67" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>140</v>
       </c>
@@ -2303,11 +2507,14 @@
       <c r="G68" t="s">
         <v>112</v>
       </c>
-      <c r="I68" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H68" t="b">
+        <v>1</v>
+      </c>
+      <c r="J68" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>143</v>
       </c>
@@ -2323,11 +2530,14 @@
       <c r="G69" t="s">
         <v>120</v>
       </c>
-      <c r="I69" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H69" t="b">
+        <v>1</v>
+      </c>
+      <c r="J69" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>145</v>
       </c>
@@ -2346,11 +2556,14 @@
       <c r="G70" t="s">
         <v>122</v>
       </c>
-      <c r="I70" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H70" t="b">
+        <v>1</v>
+      </c>
+      <c r="J70" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>148</v>
       </c>
@@ -2366,7 +2579,10 @@
       <c r="G71" t="s">
         <v>131</v>
       </c>
-      <c r="I71" t="s">
+      <c r="H71" t="b">
+        <v>1</v>
+      </c>
+      <c r="J71" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>